<commit_message>
Update Nalco data (2026-09-06 08:01:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1408"/>
+  <dimension ref="A1:H1409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -47933,6 +47933,40 @@
         <v>557</v>
       </c>
     </row>
+    <row r="1409">
+      <c r="A1409" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 08:01:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1409" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:31:04 IST</t>
+        </is>
+      </c>
+      <c r="C1409" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1409" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1409" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1409" s="1" t="inlineStr"/>
+      <c r="G1409" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1409" s="1" t="n">
+        <v>558</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-06 13:00:53 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1409"/>
+  <dimension ref="A1:H1410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -47967,6 +47967,40 @@
         <v>558</v>
       </c>
     </row>
+    <row r="1410">
+      <c r="A1410" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 13:00:47 UTC</t>
+        </is>
+      </c>
+      <c r="B1410" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:30:47 IST</t>
+        </is>
+      </c>
+      <c r="C1410" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1410" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1410" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1410" s="1" t="inlineStr"/>
+      <c r="G1410" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1410" s="1" t="n">
+        <v>558</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-07 08:31:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1410"/>
+  <dimension ref="A1:H1411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48001,6 +48001,40 @@
         <v>558</v>
       </c>
     </row>
+    <row r="1411">
+      <c r="A1411" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 08:31:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1411" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 14:01:35 IST</t>
+        </is>
+      </c>
+      <c r="C1411" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1411" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1411" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1411" s="1" t="inlineStr"/>
+      <c r="G1411" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1411" s="1" t="n">
+        <v>559</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-07 15:07:58 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1411"/>
+  <dimension ref="A1:H1412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48035,6 +48035,40 @@
         <v>559</v>
       </c>
     </row>
+    <row r="1412">
+      <c r="A1412" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 15:07:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1412" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-07 20:37:51 IST</t>
+        </is>
+      </c>
+      <c r="C1412" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1412" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1412" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2026/09/Ingot-01-09-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1412" s="1" t="inlineStr"/>
+      <c r="G1412" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1412" s="1" t="n">
+        <v>559</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-08 08:14:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1412"/>
+  <dimension ref="A1:H1413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48069,6 +48069,44 @@
         <v>559</v>
       </c>
     </row>
+    <row r="1413">
+      <c r="A1413" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 08:14:16 UTC</t>
+        </is>
+      </c>
+      <c r="B1413" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:44:16 IST</t>
+        </is>
+      </c>
+      <c r="C1413" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1413" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1413" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1413" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1413" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1413" s="1" t="n">
+        <v>560</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-08 13:45:10 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1413"/>
+  <dimension ref="A1:H1414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48107,6 +48107,40 @@
         <v>560</v>
       </c>
     </row>
+    <row r="1414">
+      <c r="A1414" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 13:45:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1414" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-08 19:15:04 IST</t>
+        </is>
+      </c>
+      <c r="C1414" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1414" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1414" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1414" s="1" t="inlineStr"/>
+      <c r="G1414" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1414" s="1" t="n">
+        <v>560</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-09 08:17:26 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1414"/>
+  <dimension ref="A1:H1415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48141,6 +48141,40 @@
         <v>560</v>
       </c>
     </row>
+    <row r="1415">
+      <c r="A1415" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 08:17:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1415" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-09 13:47:21 IST</t>
+        </is>
+      </c>
+      <c r="C1415" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1415" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1415" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-8-9-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1415" s="1" t="inlineStr"/>
+      <c r="G1415" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1415" s="1" t="n">
+        <v>561</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-15 13:05:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1415"/>
+  <dimension ref="A1:H1416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48175,6 +48175,44 @@
         <v>561</v>
       </c>
     </row>
+    <row r="1416">
+      <c r="A1416" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 13:05:48 UTC</t>
+        </is>
+      </c>
+      <c r="B1416" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 18:35:48 IST</t>
+        </is>
+      </c>
+      <c r="C1416" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1416" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1416" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1416" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1416" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1416" s="1" t="n">
+        <v>567</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-15 14:23:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1416"/>
+  <dimension ref="A1:H1417"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48213,6 +48213,40 @@
         <v>567</v>
       </c>
     </row>
+    <row r="1417">
+      <c r="A1417" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 14:23:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1417" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-15 19:53:35 IST</t>
+        </is>
+      </c>
+      <c r="C1417" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1417" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1417" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-11-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1417" s="1" t="inlineStr"/>
+      <c r="G1417" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1417" s="1" t="n">
+        <v>567</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-16 08:44:35 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1417"/>
+  <dimension ref="A1:H1418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48247,6 +48247,44 @@
         <v>567</v>
       </c>
     </row>
+    <row r="1418">
+      <c r="A1418" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 08:44:28 UTC</t>
+        </is>
+      </c>
+      <c r="B1418" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:14:28 IST</t>
+        </is>
+      </c>
+      <c r="C1418" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1418" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1418" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1418" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1418" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1418" s="1" t="n">
+        <v>568</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-16 14:16:01 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1418"/>
+  <dimension ref="A1:H1419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48285,6 +48285,40 @@
         <v>568</v>
       </c>
     </row>
+    <row r="1419">
+      <c r="A1419" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 14:15:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1419" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-16 19:45:55 IST</t>
+        </is>
+      </c>
+      <c r="C1419" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1419" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1419" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1419" s="1" t="inlineStr"/>
+      <c r="G1419" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1419" s="1" t="n">
+        <v>568</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-17 08:48:17 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1419"/>
+  <dimension ref="A1:H1420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48319,6 +48319,40 @@
         <v>568</v>
       </c>
     </row>
+    <row r="1420">
+      <c r="A1420" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 08:48:10 UTC</t>
+        </is>
+      </c>
+      <c r="B1420" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:18:10 IST</t>
+        </is>
+      </c>
+      <c r="C1420" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1420" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1420" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1420" s="1" t="inlineStr"/>
+      <c r="G1420" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1420" s="1" t="n">
+        <v>569</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-17 14:22:07 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1420"/>
+  <dimension ref="A1:H1421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48353,6 +48353,40 @@
         <v>569</v>
       </c>
     </row>
+    <row r="1421">
+      <c r="A1421" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 14:22:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1421" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-17 19:52:00 IST</t>
+        </is>
+      </c>
+      <c r="C1421" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1421" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1421" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1421" s="1" t="inlineStr"/>
+      <c r="G1421" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1421" s="1" t="n">
+        <v>569</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-18 08:24:02 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1421"/>
+  <dimension ref="A1:H1422"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48387,6 +48387,40 @@
         <v>569</v>
       </c>
     </row>
+    <row r="1422">
+      <c r="A1422" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 08:23:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1422" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:53:55 IST</t>
+        </is>
+      </c>
+      <c r="C1422" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1422" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1422" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1422" s="1" t="inlineStr"/>
+      <c r="G1422" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1422" s="1" t="n">
+        <v>570</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-18 13:42:31 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1422"/>
+  <dimension ref="A1:H1423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48421,6 +48421,40 @@
         <v>570</v>
       </c>
     </row>
+    <row r="1423">
+      <c r="A1423" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 13:42:26 UTC</t>
+        </is>
+      </c>
+      <c r="B1423" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-18 19:12:26 IST</t>
+        </is>
+      </c>
+      <c r="C1423" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1423" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1423" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1423" s="1" t="inlineStr"/>
+      <c r="G1423" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1423" s="1" t="n">
+        <v>570</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-19 08:11:34 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1423"/>
+  <dimension ref="A1:H1424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48455,6 +48455,44 @@
         <v>570</v>
       </c>
     </row>
+    <row r="1424">
+      <c r="A1424" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 08:11:28 UTC</t>
+        </is>
+      </c>
+      <c r="B1424" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 13:41:28 IST</t>
+        </is>
+      </c>
+      <c r="C1424" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1424" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1424" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1424" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1424" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1424" s="1" t="n">
+        <v>571</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-19 13:15:51 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1424"/>
+  <dimension ref="A1:H1425"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48493,6 +48493,40 @@
         <v>571</v>
       </c>
     </row>
+    <row r="1425">
+      <c r="A1425" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 13:15:45 UTC</t>
+        </is>
+      </c>
+      <c r="B1425" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-19 18:45:45 IST</t>
+        </is>
+      </c>
+      <c r="C1425" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1425" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1425" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1425" s="1" t="inlineStr"/>
+      <c r="G1425" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1425" s="1" t="n">
+        <v>571</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-20 08:44:15 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1425"/>
+  <dimension ref="A1:H1426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48527,6 +48527,40 @@
         <v>571</v>
       </c>
     </row>
+    <row r="1426">
+      <c r="A1426" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 08:44:09 UTC</t>
+        </is>
+      </c>
+      <c r="B1426" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 14:14:09 IST</t>
+        </is>
+      </c>
+      <c r="C1426" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1426" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1426" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1426" s="1" t="inlineStr"/>
+      <c r="G1426" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1426" s="1" t="n">
+        <v>572</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-20 13:38:14 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1426"/>
+  <dimension ref="A1:H1427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48561,6 +48561,40 @@
         <v>572</v>
       </c>
     </row>
+    <row r="1427">
+      <c r="A1427" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 13:38:07 UTC</t>
+        </is>
+      </c>
+      <c r="B1427" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-20 19:08:07 IST</t>
+        </is>
+      </c>
+      <c r="C1427" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1427" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1427" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1427" s="1" t="inlineStr"/>
+      <c r="G1427" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1427" s="1" t="n">
+        <v>572</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-21 09:10:51 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1427"/>
+  <dimension ref="A1:H1428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48595,6 +48595,40 @@
         <v>572</v>
       </c>
     </row>
+    <row r="1428">
+      <c r="A1428" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 09:10:44 UTC</t>
+        </is>
+      </c>
+      <c r="B1428" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 14:40:44 IST</t>
+        </is>
+      </c>
+      <c r="C1428" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1428" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1428" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1428" s="1" t="inlineStr"/>
+      <c r="G1428" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1428" s="1" t="n">
+        <v>573</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-21 15:58:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1428"/>
+  <dimension ref="A1:H1429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48629,6 +48629,40 @@
         <v>573</v>
       </c>
     </row>
+    <row r="1429">
+      <c r="A1429" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 15:58:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1429" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-21 21:28:14 IST</t>
+        </is>
+      </c>
+      <c r="C1429" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1429" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1429" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1429" s="1" t="inlineStr"/>
+      <c r="G1429" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1429" s="1" t="n">
+        <v>573</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-22 08:42:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1429"/>
+  <dimension ref="A1:H1430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48663,6 +48663,40 @@
         <v>573</v>
       </c>
     </row>
+    <row r="1430">
+      <c r="A1430" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 08:42:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1430" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:12:05 IST</t>
+        </is>
+      </c>
+      <c r="C1430" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1430" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1430" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1430" s="1" t="inlineStr"/>
+      <c r="G1430" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1430" s="1" t="n">
+        <v>574</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-22 14:06:14 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1430"/>
+  <dimension ref="A1:H1431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48697,6 +48697,40 @@
         <v>574</v>
       </c>
     </row>
+    <row r="1431">
+      <c r="A1431" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 14:06:07 UTC</t>
+        </is>
+      </c>
+      <c r="B1431" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-22 19:36:07 IST</t>
+        </is>
+      </c>
+      <c r="C1431" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1431" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1431" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1431" s="1" t="inlineStr"/>
+      <c r="G1431" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1431" s="1" t="n">
+        <v>574</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-23 08:44:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1431"/>
+  <dimension ref="A1:H1432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48731,6 +48731,40 @@
         <v>574</v>
       </c>
     </row>
+    <row r="1432">
+      <c r="A1432" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:44:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1432" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:14:14 IST</t>
+        </is>
+      </c>
+      <c r="C1432" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1432" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1432" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1432" s="1" t="inlineStr"/>
+      <c r="G1432" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1432" s="1" t="n">
+        <v>575</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-23 14:18:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1432"/>
+  <dimension ref="A1:H1433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48765,6 +48765,40 @@
         <v>575</v>
       </c>
     </row>
+    <row r="1433">
+      <c r="A1433" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:18:04 UTC</t>
+        </is>
+      </c>
+      <c r="B1433" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-23 19:48:04 IST</t>
+        </is>
+      </c>
+      <c r="C1433" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1433" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1433" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-19-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1433" s="1" t="inlineStr"/>
+      <c r="G1433" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1433" s="1" t="n">
+        <v>575</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-24 08:37:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1433"/>
+  <dimension ref="A1:H1434"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48799,6 +48799,44 @@
         <v>575</v>
       </c>
     </row>
+    <row r="1434">
+      <c r="A1434" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 08:37:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1434" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:07:30 IST</t>
+        </is>
+      </c>
+      <c r="C1434" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1434" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1434" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1434" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1434" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1434" s="1" t="n">
+        <v>576</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-24 14:16:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1434"/>
+  <dimension ref="A1:H1435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48837,6 +48837,40 @@
         <v>576</v>
       </c>
     </row>
+    <row r="1435">
+      <c r="A1435" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:16:44 UTC</t>
+        </is>
+      </c>
+      <c r="B1435" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-24 19:46:44 IST</t>
+        </is>
+      </c>
+      <c r="C1435" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1435" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1435" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1435" s="1" t="inlineStr"/>
+      <c r="G1435" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1435" s="1" t="n">
+        <v>576</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-25 08:59:18 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1435"/>
+  <dimension ref="A1:H1436"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48871,6 +48871,40 @@
         <v>576</v>
       </c>
     </row>
+    <row r="1436">
+      <c r="A1436" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 08:59:12 UTC</t>
+        </is>
+      </c>
+      <c r="B1436" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:29:12 IST</t>
+        </is>
+      </c>
+      <c r="C1436" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1436" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1436" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1436" s="1" t="inlineStr"/>
+      <c r="G1436" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1436" s="1" t="n">
+        <v>577</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-25 14:40:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1436"/>
+  <dimension ref="A1:H1437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48905,6 +48905,40 @@
         <v>577</v>
       </c>
     </row>
+    <row r="1437">
+      <c r="A1437" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:39:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1437" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-25 20:09:59 IST</t>
+        </is>
+      </c>
+      <c r="C1437" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1437" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1437" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1437" s="1" t="inlineStr"/>
+      <c r="G1437" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1437" s="1" t="n">
+        <v>577</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-26 08:45:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1437"/>
+  <dimension ref="A1:H1438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48939,6 +48939,40 @@
         <v>577</v>
       </c>
     </row>
+    <row r="1438">
+      <c r="A1438" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 08:45:02 UTC</t>
+        </is>
+      </c>
+      <c r="B1438" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 14:15:02 IST</t>
+        </is>
+      </c>
+      <c r="C1438" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1438" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1438" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1438" s="1" t="inlineStr"/>
+      <c r="G1438" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1438" s="1" t="n">
+        <v>578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-26 13:47:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1438"/>
+  <dimension ref="A1:H1439"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -48973,6 +48973,40 @@
         <v>578</v>
       </c>
     </row>
+    <row r="1439">
+      <c r="A1439" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 13:47:53 UTC</t>
+        </is>
+      </c>
+      <c r="B1439" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-26 19:17:53 IST</t>
+        </is>
+      </c>
+      <c r="C1439" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1439" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1439" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1439" s="1" t="inlineStr"/>
+      <c r="G1439" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1439" s="1" t="n">
+        <v>578</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-27 09:25:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1439"/>
+  <dimension ref="A1:H1440"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49007,6 +49007,40 @@
         <v>578</v>
       </c>
     </row>
+    <row r="1440">
+      <c r="A1440" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 09:25:34 UTC</t>
+        </is>
+      </c>
+      <c r="B1440" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:55:34 IST</t>
+        </is>
+      </c>
+      <c r="C1440" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1440" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1440" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1440" s="1" t="inlineStr"/>
+      <c r="G1440" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1440" s="1" t="n">
+        <v>579</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-27 14:46:47 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1440"/>
+  <dimension ref="A1:H1441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49041,6 +49041,40 @@
         <v>579</v>
       </c>
     </row>
+    <row r="1441">
+      <c r="A1441" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 14:46:40 UTC</t>
+        </is>
+      </c>
+      <c r="B1441" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-27 20:16:40 IST</t>
+        </is>
+      </c>
+      <c r="C1441" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1441" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1441" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1441" s="1" t="inlineStr"/>
+      <c r="G1441" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1441" s="1" t="n">
+        <v>579</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-28 10:02:18 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1441"/>
+  <dimension ref="A1:H1442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49075,6 +49075,40 @@
         <v>579</v>
       </c>
     </row>
+    <row r="1442">
+      <c r="A1442" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 10:02:12 UTC</t>
+        </is>
+      </c>
+      <c r="B1442" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:32:12 IST</t>
+        </is>
+      </c>
+      <c r="C1442" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1442" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1442" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1442" s="1" t="inlineStr"/>
+      <c r="G1442" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1442" s="1" t="n">
+        <v>580</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-28 19:46:01 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1442"/>
+  <dimension ref="A1:H1443"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49109,6 +49109,40 @@
         <v>580</v>
       </c>
     </row>
+    <row r="1443">
+      <c r="A1443" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:45:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1443" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 01:15:55 IST</t>
+        </is>
+      </c>
+      <c r="C1443" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1443" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1443" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1443" s="1" t="inlineStr"/>
+      <c r="G1443" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1443" s="1" t="n">
+        <v>581</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-29 10:01:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1443"/>
+  <dimension ref="A1:H1444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49143,6 +49143,40 @@
         <v>581</v>
       </c>
     </row>
+    <row r="1444">
+      <c r="A1444" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:00:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1444" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 15:30:59 IST</t>
+        </is>
+      </c>
+      <c r="C1444" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1444" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1444" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1444" s="1" t="inlineStr"/>
+      <c r="G1444" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1444" s="1" t="n">
+        <v>581</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-29 18:11:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1444"/>
+  <dimension ref="A1:H1445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49177,6 +49177,40 @@
         <v>581</v>
       </c>
     </row>
+    <row r="1445">
+      <c r="A1445" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:11:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1445" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-29 23:41:01 IST</t>
+        </is>
+      </c>
+      <c r="C1445" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1445" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1445" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1445" s="1" t="inlineStr"/>
+      <c r="G1445" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1445" s="1" t="n">
+        <v>581</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-30 09:53:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1445"/>
+  <dimension ref="A1:H1446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49211,6 +49211,40 @@
         <v>581</v>
       </c>
     </row>
+    <row r="1446">
+      <c r="A1446" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 09:53:51 UTC</t>
+        </is>
+      </c>
+      <c r="B1446" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:23:51 IST</t>
+        </is>
+      </c>
+      <c r="C1446" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1446" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1446" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1446" s="1" t="inlineStr"/>
+      <c r="G1446" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1446" s="1" t="n">
+        <v>582</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-09-30 18:03:06 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1446"/>
+  <dimension ref="A1:H1447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49245,6 +49245,40 @@
         <v>582</v>
       </c>
     </row>
+    <row r="1447">
+      <c r="A1447" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:03:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1447" s="1" t="inlineStr">
+        <is>
+          <t>2026-09-30 23:33:00 IST</t>
+        </is>
+      </c>
+      <c r="C1447" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1447" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1447" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1447" s="1" t="inlineStr"/>
+      <c r="G1447" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1447" s="1" t="n">
+        <v>582</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-01 10:20:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1447"/>
+  <dimension ref="A1:H1448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49279,6 +49279,40 @@
         <v>582</v>
       </c>
     </row>
+    <row r="1448">
+      <c r="A1448" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 10:20:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1448" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 15:50:35 IST</t>
+        </is>
+      </c>
+      <c r="C1448" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1448" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1448" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1448" s="1" t="inlineStr"/>
+      <c r="G1448" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1448" s="1" t="n">
+        <v>583</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-01 18:29:51 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1448"/>
+  <dimension ref="A1:H1449"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49313,6 +49313,40 @@
         <v>583</v>
       </c>
     </row>
+    <row r="1449">
+      <c r="A1449" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 18:29:45 UTC</t>
+        </is>
+      </c>
+      <c r="B1449" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-01 23:59:45 IST</t>
+        </is>
+      </c>
+      <c r="C1449" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1449" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1449" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-09-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1449" s="1" t="inlineStr"/>
+      <c r="G1449" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1449" s="1" t="n">
+        <v>583</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-02 09:57:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1449"/>
+  <dimension ref="A1:H1450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49347,6 +49347,44 @@
         <v>583</v>
       </c>
     </row>
+    <row r="1450">
+      <c r="A1450" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 09:57:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1450" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 15:27:35 IST</t>
+        </is>
+      </c>
+      <c r="C1450" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1450" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1450" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1450" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1450" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1450" s="1" t="n">
+        <v>584</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-02 17:57:26 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1450"/>
+  <dimension ref="A1:H1451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49385,6 +49385,40 @@
         <v>584</v>
       </c>
     </row>
+    <row r="1451">
+      <c r="A1451" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 17:57:20 UTC</t>
+        </is>
+      </c>
+      <c r="B1451" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-02 23:27:20 IST</t>
+        </is>
+      </c>
+      <c r="C1451" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1451" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1451" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1451" s="1" t="inlineStr"/>
+      <c r="G1451" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1451" s="1" t="n">
+        <v>584</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-03 09:19:41 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1451"/>
+  <dimension ref="A1:H1452"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49419,6 +49419,40 @@
         <v>584</v>
       </c>
     </row>
+    <row r="1452">
+      <c r="A1452" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 09:19:35 UTC</t>
+        </is>
+      </c>
+      <c r="B1452" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:49:35 IST</t>
+        </is>
+      </c>
+      <c r="C1452" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1452" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1452" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1452" s="1" t="inlineStr"/>
+      <c r="G1452" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1452" s="1" t="n">
+        <v>585</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-03 14:22:07 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1452"/>
+  <dimension ref="A1:H1453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49453,6 +49453,40 @@
         <v>585</v>
       </c>
     </row>
+    <row r="1453">
+      <c r="A1453" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 14:22:02 UTC</t>
+        </is>
+      </c>
+      <c r="B1453" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-03 19:52:02 IST</t>
+        </is>
+      </c>
+      <c r="C1453" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1453" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1453" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1453" s="1" t="inlineStr"/>
+      <c r="G1453" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1453" s="1" t="n">
+        <v>585</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-04 09:59:01 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1453"/>
+  <dimension ref="A1:H1454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49487,6 +49487,40 @@
         <v>585</v>
       </c>
     </row>
+    <row r="1454">
+      <c r="A1454" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 09:58:55 UTC</t>
+        </is>
+      </c>
+      <c r="B1454" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 15:28:55 IST</t>
+        </is>
+      </c>
+      <c r="C1454" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1454" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1454" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1454" s="1" t="inlineStr"/>
+      <c r="G1454" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1454" s="1" t="n">
+        <v>586</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-04 16:55:17 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1454"/>
+  <dimension ref="A1:H1455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49521,6 +49521,40 @@
         <v>586</v>
       </c>
     </row>
+    <row r="1455">
+      <c r="A1455" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 16:55:12 UTC</t>
+        </is>
+      </c>
+      <c r="B1455" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-04 22:25:12 IST</t>
+        </is>
+      </c>
+      <c r="C1455" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1455" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1455" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1455" s="1" t="inlineStr"/>
+      <c r="G1455" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1455" s="1" t="n">
+        <v>586</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-05 10:43:20 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1455"/>
+  <dimension ref="A1:H1456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49555,6 +49555,40 @@
         <v>586</v>
       </c>
     </row>
+    <row r="1456">
+      <c r="A1456" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05 10:43:13 UTC</t>
+        </is>
+      </c>
+      <c r="B1456" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05 16:13:13 IST</t>
+        </is>
+      </c>
+      <c r="C1456" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1456" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1456" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1456" s="1" t="inlineStr"/>
+      <c r="G1456" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1456" s="1" t="n">
+        <v>587</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-05 20:37:56 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1456"/>
+  <dimension ref="A1:H1457"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49589,6 +49589,40 @@
         <v>587</v>
       </c>
     </row>
+    <row r="1457">
+      <c r="A1457" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05 20:37:48 UTC</t>
+        </is>
+      </c>
+      <c r="B1457" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 02:07:48 IST</t>
+        </is>
+      </c>
+      <c r="C1457" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1457" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1457" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1457" s="1" t="inlineStr"/>
+      <c r="G1457" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1457" s="1" t="n">
+        <v>588</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-06 10:36:25 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1457"/>
+  <dimension ref="A1:H1458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49623,6 +49623,40 @@
         <v>588</v>
       </c>
     </row>
+    <row r="1458">
+      <c r="A1458" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 10:36:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1458" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 16:06:18 IST</t>
+        </is>
+      </c>
+      <c r="C1458" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1458" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1458" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1458" s="1" t="inlineStr"/>
+      <c r="G1458" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1458" s="1" t="n">
+        <v>588</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-06 18:31:09 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1458"/>
+  <dimension ref="A1:H1459"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49657,6 +49657,40 @@
         <v>588</v>
       </c>
     </row>
+    <row r="1459">
+      <c r="A1459" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:31:03 UTC</t>
+        </is>
+      </c>
+      <c r="B1459" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 00:01:03 IST</t>
+        </is>
+      </c>
+      <c r="C1459" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1459" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1459" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1459" s="1" t="inlineStr"/>
+      <c r="G1459" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1459" s="1" t="n">
+        <v>589</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-07 10:27:46 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1459"/>
+  <dimension ref="A1:H1460"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49691,6 +49691,40 @@
         <v>589</v>
       </c>
     </row>
+    <row r="1460">
+      <c r="A1460" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 10:27:39 UTC</t>
+        </is>
+      </c>
+      <c r="B1460" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 15:57:39 IST</t>
+        </is>
+      </c>
+      <c r="C1460" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1460" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1460" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1460" s="1" t="inlineStr"/>
+      <c r="G1460" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1460" s="1" t="n">
+        <v>589</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-07 19:01:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1460"/>
+  <dimension ref="A1:H1461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49725,6 +49725,40 @@
         <v>589</v>
       </c>
     </row>
+    <row r="1461">
+      <c r="A1461" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:00:56 UTC</t>
+        </is>
+      </c>
+      <c r="B1461" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 00:30:56 IST</t>
+        </is>
+      </c>
+      <c r="C1461" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1461" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1461" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1461" s="1" t="inlineStr"/>
+      <c r="G1461" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1461" s="1" t="n">
+        <v>590</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-08 10:48:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1461"/>
+  <dimension ref="A1:H1462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49759,6 +49759,40 @@
         <v>590</v>
       </c>
     </row>
+    <row r="1462">
+      <c r="A1462" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 10:48:19 UTC</t>
+        </is>
+      </c>
+      <c r="B1462" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 16:18:19 IST</t>
+        </is>
+      </c>
+      <c r="C1462" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1462" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1462" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1462" s="1" t="inlineStr"/>
+      <c r="G1462" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1462" s="1" t="n">
+        <v>590</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-08 18:56:30 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1462"/>
+  <dimension ref="A1:H1463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49793,6 +49793,40 @@
         <v>590</v>
       </c>
     </row>
+    <row r="1463">
+      <c r="A1463" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-08 18:56:23 UTC</t>
+        </is>
+      </c>
+      <c r="B1463" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 00:26:23 IST</t>
+        </is>
+      </c>
+      <c r="C1463" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1463" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1463" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1463" s="1" t="inlineStr"/>
+      <c r="G1463" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1463" s="1" t="n">
+        <v>591</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-09 10:47:20 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1463"/>
+  <dimension ref="A1:H1464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49827,6 +49827,40 @@
         <v>591</v>
       </c>
     </row>
+    <row r="1464">
+      <c r="A1464" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 10:47:13 UTC</t>
+        </is>
+      </c>
+      <c r="B1464" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 16:17:13 IST</t>
+        </is>
+      </c>
+      <c r="C1464" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1464" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1464" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1464" s="1" t="inlineStr"/>
+      <c r="G1464" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1464" s="1" t="n">
+        <v>591</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-09 18:26:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1464"/>
+  <dimension ref="A1:H1465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49861,6 +49861,40 @@
         <v>591</v>
       </c>
     </row>
+    <row r="1465">
+      <c r="A1465" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:26:36 UTC</t>
+        </is>
+      </c>
+      <c r="B1465" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-09 23:56:36 IST</t>
+        </is>
+      </c>
+      <c r="C1465" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1465" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1465" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1465" s="1" t="inlineStr"/>
+      <c r="G1465" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1465" s="1" t="n">
+        <v>591</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-10 10:02:26 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1465"/>
+  <dimension ref="A1:H1466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49895,6 +49895,40 @@
         <v>591</v>
       </c>
     </row>
+    <row r="1466">
+      <c r="A1466" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 10:02:17 UTC</t>
+        </is>
+      </c>
+      <c r="B1466" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 15:32:17 IST</t>
+        </is>
+      </c>
+      <c r="C1466" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1466" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1466" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1466" s="1" t="inlineStr"/>
+      <c r="G1466" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1466" s="1" t="n">
+        <v>592</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-10 17:24:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1466"/>
+  <dimension ref="A1:H1467"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49929,6 +49929,40 @@
         <v>592</v>
       </c>
     </row>
+    <row r="1467">
+      <c r="A1467" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 17:24:44 UTC</t>
+        </is>
+      </c>
+      <c r="B1467" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-10 22:54:44 IST</t>
+        </is>
+      </c>
+      <c r="C1467" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1467" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1467" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1467" s="1" t="inlineStr"/>
+      <c r="G1467" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1467" s="1" t="n">
+        <v>592</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-11 10:12:24 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1467"/>
+  <dimension ref="A1:H1468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49963,6 +49963,40 @@
         <v>592</v>
       </c>
     </row>
+    <row r="1468">
+      <c r="A1468" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 10:12:17 UTC</t>
+        </is>
+      </c>
+      <c r="B1468" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 15:42:17 IST</t>
+        </is>
+      </c>
+      <c r="C1468" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1468" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1468" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1468" s="1" t="inlineStr"/>
+      <c r="G1468" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1468" s="1" t="n">
+        <v>593</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-11 17:44:03 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1468"/>
+  <dimension ref="A1:H1469"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -49997,6 +49997,40 @@
         <v>593</v>
       </c>
     </row>
+    <row r="1469">
+      <c r="A1469" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 17:43:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1469" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:13:58 IST</t>
+        </is>
+      </c>
+      <c r="C1469" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1469" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1469" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1469" s="1" t="inlineStr"/>
+      <c r="G1469" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1469" s="1" t="n">
+        <v>593</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-12 11:10:54 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1469"/>
+  <dimension ref="A1:H1470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50031,6 +50031,40 @@
         <v>593</v>
       </c>
     </row>
+    <row r="1470">
+      <c r="A1470" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 11:10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B1470" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 16:40:48 IST</t>
+        </is>
+      </c>
+      <c r="C1470" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1470" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1470" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1470" s="1" t="inlineStr"/>
+      <c r="G1470" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1470" s="1" t="n">
+        <v>594</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-12 21:20:39 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1470"/>
+  <dimension ref="A1:H1471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50065,6 +50065,40 @@
         <v>594</v>
       </c>
     </row>
+    <row r="1471">
+      <c r="A1471" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-12 21:20:34 UTC</t>
+        </is>
+      </c>
+      <c r="B1471" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 02:50:34 IST</t>
+        </is>
+      </c>
+      <c r="C1471" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1471" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1471" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-01-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1471" s="1" t="inlineStr"/>
+      <c r="G1471" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1471" s="1" t="n">
+        <v>595</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-13 10:52:22 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1471"/>
+  <dimension ref="A1:H1472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50099,6 +50099,44 @@
         <v>595</v>
       </c>
     </row>
+    <row r="1472">
+      <c r="A1472" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 10:52:16 UTC</t>
+        </is>
+      </c>
+      <c r="B1472" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 16:22:16 IST</t>
+        </is>
+      </c>
+      <c r="C1472" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1472" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1472" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1472" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1472" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1472" s="1" t="n">
+        <v>595</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-13 19:25:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1472"/>
+  <dimension ref="A1:H1473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50137,6 +50137,40 @@
         <v>595</v>
       </c>
     </row>
+    <row r="1473">
+      <c r="A1473" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:24:59 UTC</t>
+        </is>
+      </c>
+      <c r="B1473" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 00:54:59 IST</t>
+        </is>
+      </c>
+      <c r="C1473" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1473" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1473" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1473" s="1" t="inlineStr"/>
+      <c r="G1473" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1473" s="1" t="n">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-14 08:54:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1473"/>
+  <dimension ref="A1:H1474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50171,6 +50171,40 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1474">
+      <c r="A1474" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 08:54:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1474" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:24:05 IST</t>
+        </is>
+      </c>
+      <c r="C1474" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1474" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1474" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1474" s="1" t="inlineStr"/>
+      <c r="G1474" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1474" s="1" t="n">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-14 14:35:30 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1474"/>
+  <dimension ref="A1:H1475"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50205,6 +50205,40 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1475">
+      <c r="A1475" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:35:23 UTC</t>
+        </is>
+      </c>
+      <c r="B1475" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14 20:05:23 IST</t>
+        </is>
+      </c>
+      <c r="C1475" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1475" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1475" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1475" s="1" t="inlineStr"/>
+      <c r="G1475" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1475" s="1" t="n">
+        <v>596</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-15 08:29:00 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1475"/>
+  <dimension ref="A1:H1476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50239,6 +50239,40 @@
         <v>596</v>
       </c>
     </row>
+    <row r="1476">
+      <c r="A1476" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 08:28:53 UTC</t>
+        </is>
+      </c>
+      <c r="B1476" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 13:58:53 IST</t>
+        </is>
+      </c>
+      <c r="C1476" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1476" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1476" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1476" s="1" t="inlineStr"/>
+      <c r="G1476" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1476" s="1" t="n">
+        <v>597</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-15 14:16:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1476"/>
+  <dimension ref="A1:H1477"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50273,6 +50273,40 @@
         <v>597</v>
       </c>
     </row>
+    <row r="1477">
+      <c r="A1477" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 14:16:06 UTC</t>
+        </is>
+      </c>
+      <c r="B1477" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-15 19:46:06 IST</t>
+        </is>
+      </c>
+      <c r="C1477" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1477" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1477" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-13-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1477" s="1" t="inlineStr"/>
+      <c r="G1477" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1477" s="1" t="n">
+        <v>597</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-16 08:21:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1477"/>
+  <dimension ref="A1:H1478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50307,6 +50307,44 @@
         <v>597</v>
       </c>
     </row>
+    <row r="1478">
+      <c r="A1478" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 08:21:49 UTC</t>
+        </is>
+      </c>
+      <c r="B1478" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:51:49 IST</t>
+        </is>
+      </c>
+      <c r="C1478" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1478" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1478" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1478" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="G1478" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1478" s="1" t="n">
+        <v>598</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-16 14:05:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1478"/>
+  <dimension ref="A1:H1479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50345,6 +50345,40 @@
         <v>598</v>
       </c>
     </row>
+    <row r="1479">
+      <c r="A1479" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 14:05:14 UTC</t>
+        </is>
+      </c>
+      <c r="B1479" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-16 19:35:14 IST</t>
+        </is>
+      </c>
+      <c r="C1479" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1479" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1479" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1479" s="1" t="inlineStr"/>
+      <c r="G1479" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1479" s="1" t="n">
+        <v>598</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-17 07:57:11 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1479"/>
+  <dimension ref="A1:H1480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50379,6 +50379,40 @@
         <v>598</v>
       </c>
     </row>
+    <row r="1480">
+      <c r="A1480" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 07:57:06 UTC</t>
+        </is>
+      </c>
+      <c r="B1480" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:27:06 IST</t>
+        </is>
+      </c>
+      <c r="C1480" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1480" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1480" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1480" s="1" t="inlineStr"/>
+      <c r="G1480" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1480" s="1" t="n">
+        <v>599</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-17 13:04:25 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1480"/>
+  <dimension ref="A1:H1481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50413,6 +50413,40 @@
         <v>599</v>
       </c>
     </row>
+    <row r="1481">
+      <c r="A1481" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 13:04:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1481" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-17 18:34:18 IST</t>
+        </is>
+      </c>
+      <c r="C1481" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1481" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1481" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1481" s="1" t="inlineStr"/>
+      <c r="G1481" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1481" s="1" t="n">
+        <v>599</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-18 08:12:21 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1481"/>
+  <dimension ref="A1:H1482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50447,6 +50447,40 @@
         <v>599</v>
       </c>
     </row>
+    <row r="1482">
+      <c r="A1482" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 08:12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B1482" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:42:15 IST</t>
+        </is>
+      </c>
+      <c r="C1482" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1482" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1482" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1482" s="1" t="inlineStr"/>
+      <c r="G1482" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1482" s="1" t="n">
+        <v>600</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-18 13:24:19 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1482"/>
+  <dimension ref="A1:H1483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50481,6 +50481,40 @@
         <v>600</v>
       </c>
     </row>
+    <row r="1483">
+      <c r="A1483" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 13:24:13 UTC</t>
+        </is>
+      </c>
+      <c r="B1483" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-18 18:54:13 IST</t>
+        </is>
+      </c>
+      <c r="C1483" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1483" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1483" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1483" s="1" t="inlineStr"/>
+      <c r="G1483" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1483" s="1" t="n">
+        <v>600</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-19 09:09:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1483"/>
+  <dimension ref="A1:H1484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50515,6 +50515,40 @@
         <v>600</v>
       </c>
     </row>
+    <row r="1484">
+      <c r="A1484" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 09:09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B1484" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 14:39:42 IST</t>
+        </is>
+      </c>
+      <c r="C1484" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1484" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1484" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1484" s="1" t="inlineStr"/>
+      <c r="G1484" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1484" s="1" t="n">
+        <v>601</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-19 16:33:59 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1484"/>
+  <dimension ref="A1:H1485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50549,6 +50549,40 @@
         <v>601</v>
       </c>
     </row>
+    <row r="1485">
+      <c r="A1485" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 16:33:54 UTC</t>
+        </is>
+      </c>
+      <c r="B1485" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-19 22:03:54 IST</t>
+        </is>
+      </c>
+      <c r="C1485" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1485" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1485" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1485" s="1" t="inlineStr"/>
+      <c r="G1485" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1485" s="1" t="n">
+        <v>601</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-20 08:45:25 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1485"/>
+  <dimension ref="A1:H1486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50583,6 +50583,40 @@
         <v>601</v>
       </c>
     </row>
+    <row r="1486">
+      <c r="A1486" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 08:45:21 UTC</t>
+        </is>
+      </c>
+      <c r="B1486" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:15:21 IST</t>
+        </is>
+      </c>
+      <c r="C1486" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1486" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1486" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1486" s="1" t="inlineStr"/>
+      <c r="G1486" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1486" s="1" t="n">
+        <v>602</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-20 14:24:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1486"/>
+  <dimension ref="A1:H1487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50617,6 +50617,40 @@
         <v>602</v>
       </c>
     </row>
+    <row r="1487">
+      <c r="A1487" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 14:23:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1487" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:53:58 IST</t>
+        </is>
+      </c>
+      <c r="C1487" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1487" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1487" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1487" s="1" t="inlineStr"/>
+      <c r="G1487" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1487" s="1" t="n">
+        <v>602</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-21 08:45:43 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1487"/>
+  <dimension ref="A1:H1488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50651,6 +50651,40 @@
         <v>602</v>
       </c>
     </row>
+    <row r="1488">
+      <c r="A1488" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 08:45:37 UTC</t>
+        </is>
+      </c>
+      <c r="B1488" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:15:37 IST</t>
+        </is>
+      </c>
+      <c r="C1488" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1488" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1488" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1488" s="1" t="inlineStr"/>
+      <c r="G1488" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1488" s="1" t="n">
+        <v>603</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-21 14:33:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1488"/>
+  <dimension ref="A1:H1489"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50685,6 +50685,40 @@
         <v>603</v>
       </c>
     </row>
+    <row r="1489">
+      <c r="A1489" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 14:33:30 UTC</t>
+        </is>
+      </c>
+      <c r="B1489" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-21 20:03:30 IST</t>
+        </is>
+      </c>
+      <c r="C1489" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1489" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1489" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1489" s="1" t="inlineStr"/>
+      <c r="G1489" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1489" s="1" t="n">
+        <v>603</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-22 08:48:05 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1489"/>
+  <dimension ref="A1:H1490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50719,6 +50719,40 @@
         <v>603</v>
       </c>
     </row>
+    <row r="1490">
+      <c r="A1490" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 08:47:58 UTC</t>
+        </is>
+      </c>
+      <c r="B1490" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:17:58 IST</t>
+        </is>
+      </c>
+      <c r="C1490" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1490" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1490" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1490" s="1" t="inlineStr"/>
+      <c r="G1490" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1490" s="1" t="n">
+        <v>604</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-22 14:35:06 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1490"/>
+  <dimension ref="A1:H1491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50753,6 +50753,40 @@
         <v>604</v>
       </c>
     </row>
+    <row r="1491">
+      <c r="A1491" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 14:35:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1491" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-22 20:05:00 IST</t>
+        </is>
+      </c>
+      <c r="C1491" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1491" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1491" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1491" s="1" t="inlineStr"/>
+      <c r="G1491" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1491" s="1" t="n">
+        <v>604</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-23 08:43:49 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1491"/>
+  <dimension ref="A1:H1492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50787,6 +50787,40 @@
         <v>604</v>
       </c>
     </row>
+    <row r="1492">
+      <c r="A1492" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 08:43:41 UTC</t>
+        </is>
+      </c>
+      <c r="B1492" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:13:41 IST</t>
+        </is>
+      </c>
+      <c r="C1492" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1492" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1492" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1492" s="1" t="inlineStr"/>
+      <c r="G1492" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1492" s="1" t="n">
+        <v>605</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-23 14:19:30 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1492"/>
+  <dimension ref="A1:H1493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50821,6 +50821,40 @@
         <v>605</v>
       </c>
     </row>
+    <row r="1493">
+      <c r="A1493" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 14:19:24 UTC</t>
+        </is>
+      </c>
+      <c r="B1493" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-23 19:49:24 IST</t>
+        </is>
+      </c>
+      <c r="C1493" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1493" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1493" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-16-10-2026.pdf</t>
+        </is>
+      </c>
+      <c r="F1493" s="1" t="inlineStr"/>
+      <c r="G1493" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1493" s="1" t="n">
+        <v>605</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-24 08:18:23 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1493"/>
+  <dimension ref="A1:H1494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50855,6 +50855,44 @@
         <v>605</v>
       </c>
     </row>
+    <row r="1494">
+      <c r="A1494" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 08:18:16 UTC</t>
+        </is>
+      </c>
+      <c r="B1494" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:48:16 IST</t>
+        </is>
+      </c>
+      <c r="C1494" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1494" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1494" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1494" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="G1494" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1494" s="1" t="n">
+        <v>606</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-24 13:26:42 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1494"/>
+  <dimension ref="A1:H1495"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50893,6 +50893,40 @@
         <v>606</v>
       </c>
     </row>
+    <row r="1495">
+      <c r="A1495" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 13:26:37 UTC</t>
+        </is>
+      </c>
+      <c r="B1495" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:56:37 IST</t>
+        </is>
+      </c>
+      <c r="C1495" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1495" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1495" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1495" s="1" t="inlineStr"/>
+      <c r="G1495" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1495" s="1" t="n">
+        <v>606</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-25 08:36:52 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1495"/>
+  <dimension ref="A1:H1496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50927,6 +50927,40 @@
         <v>606</v>
       </c>
     </row>
+    <row r="1496">
+      <c r="A1496" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 08:36:44 UTC</t>
+        </is>
+      </c>
+      <c r="B1496" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 14:06:44 IST</t>
+        </is>
+      </c>
+      <c r="C1496" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1496" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1496" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1496" s="1" t="inlineStr"/>
+      <c r="G1496" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1496" s="1" t="n">
+        <v>607</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-25 13:48:25 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1496"/>
+  <dimension ref="A1:H1497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50961,6 +50961,40 @@
         <v>607</v>
       </c>
     </row>
+    <row r="1497">
+      <c r="A1497" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 13:48:18 UTC</t>
+        </is>
+      </c>
+      <c r="B1497" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-25 19:18:18 IST</t>
+        </is>
+      </c>
+      <c r="C1497" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1497" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1497" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1497" s="1" t="inlineStr"/>
+      <c r="G1497" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1497" s="1" t="n">
+        <v>607</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-26 09:12:53 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1497"/>
+  <dimension ref="A1:H1498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -50995,6 +50995,40 @@
         <v>607</v>
       </c>
     </row>
+    <row r="1498">
+      <c r="A1498" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 09:12:46 UTC</t>
+        </is>
+      </c>
+      <c r="B1498" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 14:42:46 IST</t>
+        </is>
+      </c>
+      <c r="C1498" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1498" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1498" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1498" s="1" t="inlineStr"/>
+      <c r="G1498" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1498" s="1" t="n">
+        <v>608</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-26 16:13:55 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1498"/>
+  <dimension ref="A1:H1499"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51029,6 +51029,40 @@
         <v>608</v>
       </c>
     </row>
+    <row r="1499">
+      <c r="A1499" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 16:13:50 UTC</t>
+        </is>
+      </c>
+      <c r="B1499" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-26 21:43:50 IST</t>
+        </is>
+      </c>
+      <c r="C1499" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1499" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1499" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1499" s="1" t="inlineStr"/>
+      <c r="G1499" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1499" s="1" t="n">
+        <v>608</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-27 09:13:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1499"/>
+  <dimension ref="A1:H1500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51063,6 +51063,40 @@
         <v>608</v>
       </c>
     </row>
+    <row r="1500">
+      <c r="A1500" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 09:13:31 UTC</t>
+        </is>
+      </c>
+      <c r="B1500" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 14:43:31 IST</t>
+        </is>
+      </c>
+      <c r="C1500" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1500" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1500" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1500" s="1" t="inlineStr"/>
+      <c r="G1500" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1500" s="1" t="n">
+        <v>609</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-27 15:28:04 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1500"/>
+  <dimension ref="A1:H1501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51097,6 +51097,40 @@
         <v>609</v>
       </c>
     </row>
+    <row r="1501">
+      <c r="A1501" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 15:28:00 UTC</t>
+        </is>
+      </c>
+      <c r="B1501" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-27 20:58:00 IST</t>
+        </is>
+      </c>
+      <c r="C1501" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1501" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1501" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1501" s="1" t="inlineStr"/>
+      <c r="G1501" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1501" s="1" t="n">
+        <v>609</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-28 09:54:30 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1501"/>
+  <dimension ref="A1:H1502"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51131,6 +51131,40 @@
         <v>609</v>
       </c>
     </row>
+    <row r="1502">
+      <c r="A1502" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 09:54:24 UTC</t>
+        </is>
+      </c>
+      <c r="B1502" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 15:24:24 IST</t>
+        </is>
+      </c>
+      <c r="C1502" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1502" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1502" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1502" s="1" t="inlineStr"/>
+      <c r="G1502" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1502" s="1" t="n">
+        <v>610</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-28 18:24:50 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1502"/>
+  <dimension ref="A1:H1503"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51165,6 +51165,40 @@
         <v>610</v>
       </c>
     </row>
+    <row r="1503">
+      <c r="A1503" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:24:45 UTC</t>
+        </is>
+      </c>
+      <c r="B1503" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-28 23:54:45 IST</t>
+        </is>
+      </c>
+      <c r="C1503" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1503" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1503" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-24-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1503" s="1" t="inlineStr"/>
+      <c r="G1503" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1503" s="1" t="n">
+        <v>610</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-29 10:16:40 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1503"/>
+  <dimension ref="A1:H1504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51199,6 +51199,44 @@
         <v>610</v>
       </c>
     </row>
+    <row r="1504">
+      <c r="A1504" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-29 10:16:31 UTC</t>
+        </is>
+      </c>
+      <c r="B1504" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-29 15:46:31 IST</t>
+        </is>
+      </c>
+      <c r="C1504" s="1" t="inlineStr">
+        <is>
+          <t>UPDATED</t>
+        </is>
+      </c>
+      <c r="D1504" s="1" t="inlineStr">
+        <is>
+          <t>New circular processed and daily sheet rebuilt.</t>
+        </is>
+      </c>
+      <c r="E1504" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1504" s="1" t="inlineStr">
+        <is>
+          <t>/home/runner/work/nalco_circular_downloader/nalco_circular_downloader/pdfs/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="G1504" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H1504" s="1" t="n">
+        <v>611</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-29 18:34:36 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1504"/>
+  <dimension ref="A1:H1505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51237,6 +51237,40 @@
         <v>611</v>
       </c>
     </row>
+    <row r="1505">
+      <c r="A1505" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:34:29 UTC</t>
+        </is>
+      </c>
+      <c r="B1505" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 00:04:29 IST</t>
+        </is>
+      </c>
+      <c r="C1505" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1505" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1505" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1505" s="1" t="inlineStr"/>
+      <c r="G1505" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1505" s="1" t="n">
+        <v>612</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-30 10:18:17 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1505"/>
+  <dimension ref="A1:H1506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51271,6 +51271,40 @@
         <v>612</v>
       </c>
     </row>
+    <row r="1506">
+      <c r="A1506" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 10:18:11 UTC</t>
+        </is>
+      </c>
+      <c r="B1506" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 15:48:11 IST</t>
+        </is>
+      </c>
+      <c r="C1506" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1506" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1506" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1506" s="1" t="inlineStr"/>
+      <c r="G1506" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1506" s="1" t="n">
+        <v>612</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-30 18:06:38 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1506"/>
+  <dimension ref="A1:H1507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51305,6 +51305,40 @@
         <v>612</v>
       </c>
     </row>
+    <row r="1507">
+      <c r="A1507" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:06:33 UTC</t>
+        </is>
+      </c>
+      <c r="B1507" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-30 23:36:33 IST</t>
+        </is>
+      </c>
+      <c r="C1507" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1507" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1507" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1507" s="1" t="inlineStr"/>
+      <c r="G1507" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1507" s="1" t="n">
+        <v>612</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-31 09:51:27 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1507"/>
+  <dimension ref="A1:H1508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51339,6 +51339,40 @@
         <v>612</v>
       </c>
     </row>
+    <row r="1508">
+      <c r="A1508" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 09:51:20 UTC</t>
+        </is>
+      </c>
+      <c r="B1508" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 15:21:20 IST</t>
+        </is>
+      </c>
+      <c r="C1508" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1508" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1508" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1508" s="1" t="inlineStr"/>
+      <c r="G1508" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1508" s="1" t="n">
+        <v>613</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Nalco data (2026-10-31 17:18:12 UTC)
</commit_message>
<xml_diff>
--- a/data/nalco_run_log.xlsx
+++ b/data/nalco_run_log.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1508"/>
+  <dimension ref="A1:H1509"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -51373,6 +51373,40 @@
         <v>613</v>
       </c>
     </row>
+    <row r="1509">
+      <c r="A1509" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 17:18:07 UTC</t>
+        </is>
+      </c>
+      <c r="B1509" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-31 22:48:07 IST</t>
+        </is>
+      </c>
+      <c r="C1509" s="1" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="D1509" s="1" t="inlineStr">
+        <is>
+          <t>No change in PDF. Rebuilding daily sheet up to yesterday.</t>
+        </is>
+      </c>
+      <c r="E1509" s="1" t="inlineStr">
+        <is>
+          <t>https://nalcoindia.com/wp-content/uploads/2019/01/Ingot-29-10-26.pdf</t>
+        </is>
+      </c>
+      <c r="F1509" s="1" t="inlineStr"/>
+      <c r="G1509" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H1509" s="1" t="n">
+        <v>613</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>